<commit_message>
Make network deals the growth engine in CX model
Network launches ramp $20M/$40M/$60M/$70M/$80M (signed ~$70M book, then
>$700M pipeline); micro/paratransit growth slows to 10%->6% after FY26.
Adds network % of revenue and share of revenue growth rows. Network is
~36% of FY27 growth and 26% of FY30 revenue; GM falls to 36.7%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SeH2hRmBJJDZz9MSQAPubz
</commit_message>
<xml_diff>
--- a/model/CX_VIA_Model.xlsx
+++ b/model/CX_VIA_Model.xlsx
@@ -1430,57 +1430,57 @@
         <t>Historical total revenue links to Annual IS (CapIQ).</t>
       </text>
     </comment>
-    <comment ref="F17" authorId="0" shapeId="0">
+    <comment ref="F19" authorId="0" shapeId="0">
       <text>
         <t>Organic customer growth ~9% ex-Downtowner (thesis 3), ~+2%/yr price. FY26 +3%: 94 small Downtowner customers add little. Software fees face near-zero bids (Spare bid $0.01 at LA Metro).</t>
       </text>
     </comment>
-    <comment ref="F18" authorId="0" shapeId="0">
+    <comment ref="F20" authorId="0" shapeId="0">
       <text>
-        <t>Expansion at existing customers less budget-driven downsell (~4%/yr: Jersey City cut ~half, federal stopgap / ARPA cliff), with price +2%/yr as rebids reset rates. FY26 +28% ties to 1H26 actuals ($263M revenue) plus the H2 ramp.</t>
+        <t>Pilots are budget-bound (thesis 3): expansion at existing customers less downsell (Jersey City cut ~half; federal stopgap / ARPA cliff), price +2%/yr as rebids reset rates. Growth shifts to network deals. FY26 +28% ties to 1H26 actuals ($263M revenue) plus the H2 ramp.</t>
       </text>
     </comment>
-    <comment ref="F19" authorId="0" shapeId="0">
+    <comment ref="F21" authorId="0" shapeId="0">
       <text>
-        <t>FY26: Twin Cities MI (Apr), Rochester $14.6M (Sep) and part of the 2026 wins; FY27: rest of the signed ~$70M book. Then ~2 mid-sized cities a year (thesis 1.1). Earned at half rate in the launch year.</t>
+        <t>The growth engine (thesis 1). FY26: Twin Cities MI (Apr), Rochester $14.6M (Sep), part of the 2026 wins. FY27: rest of the signed ~$70M book (~$27M) plus new wins. FY28+: the &gt;$700M pipeline (doubled YoY) converting at ~8-11% a year, ~5-7 mid-sized cities at $10-15M each. Earned at half rate in the launch year.</t>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0">
+    <comment ref="D22" authorId="0" shapeId="0">
       <text>
         <t>Sioux Falls: 2024 NTD purchased transportation paid $11.07M (Via's first network deal).</t>
       </text>
     </comment>
-    <comment ref="E20" authorId="0" shapeId="0">
+    <comment ref="E22" authorId="0" shapeId="0">
       <text>
         <t>Sioux Falls ~$11.4M + Mobile $12.1M/yr (from Oct 2025).</t>
       </text>
     </comment>
-    <comment ref="E21" authorId="0" shapeId="0">
+    <comment ref="E23" authorId="0" shapeId="0">
       <text>
         <t>10-K: one-time revenue 3% of total in FY24 and FY25 (97% recurring). FY23 assumed the same.</t>
       </text>
     </comment>
-    <comment ref="F21" authorId="0" shapeId="0">
+    <comment ref="F23" authorId="0" shapeId="0">
       <text>
         <t>3% (10-K FY24-25; 1H26 also 3%).</t>
       </text>
     </comment>
-    <comment ref="F24" authorId="0" shapeId="0">
+    <comment ref="F26" authorId="0" shapeId="0">
       <text>
         <t>Bleecker assumption; reported cost split implies ~73%.</t>
       </text>
     </comment>
-    <comment ref="F25" authorId="0" shapeId="0">
+    <comment ref="F27" authorId="0" shapeId="0">
       <text>
         <t>Bleecker TaaS gross margin, arithmetic corrected and updated to 2026 contract pricing.</t>
       </text>
     </comment>
-    <comment ref="F26" authorId="0" shapeId="0">
+    <comment ref="F28" authorId="0" shapeId="0">
       <text>
         <t>ASSUMPTION (undisclosed): operator economics, below the ~29% on microtransit. Labor is 72% of mid-sized bus system cost (NTD 2024); CFO: 'some accretive, some less.'</t>
       </text>
     </comment>
-    <comment ref="F27" authorId="0" shapeId="0">
+    <comment ref="F29" authorId="0" shapeId="0">
       <text>
         <t>Implementation / consulting.</t>
       </text>
@@ -2945,23 +2945,23 @@
         <v/>
       </c>
       <c r="F32" s="257">
-        <f>1-'Revenue Build'!F29</f>
+        <f>1-'Revenue Build'!F31</f>
         <v/>
       </c>
       <c r="G32" s="258">
-        <f>1-'Revenue Build'!G29</f>
+        <f>1-'Revenue Build'!G31</f>
         <v/>
       </c>
       <c r="H32" s="258">
-        <f>1-'Revenue Build'!H29</f>
+        <f>1-'Revenue Build'!H31</f>
         <v/>
       </c>
       <c r="I32" s="258">
-        <f>1-'Revenue Build'!I29</f>
+        <f>1-'Revenue Build'!I31</f>
         <v/>
       </c>
       <c r="J32" s="258">
-        <f>1-'Revenue Build'!J29</f>
+        <f>1-'Revenue Build'!J31</f>
         <v/>
       </c>
       <c r="L32" s="13" t="inlineStr">
@@ -5588,23 +5588,23 @@
         <v>101.1</v>
       </c>
       <c r="F4" s="276">
-        <f>E4*(1+F17)</f>
+        <f>E4*(1+F19)</f>
         <v/>
       </c>
       <c r="G4" s="276">
-        <f>F4*(1+G17)</f>
+        <f>F4*(1+G19)</f>
         <v/>
       </c>
       <c r="H4" s="276">
-        <f>G4*(1+H17)</f>
+        <f>G4*(1+H19)</f>
         <v/>
       </c>
       <c r="I4" s="276">
-        <f>H4*(1+I17)</f>
+        <f>H4*(1+I19)</f>
         <v/>
       </c>
       <c r="J4" s="276">
-        <f>I4*(1+J17)</f>
+        <f>I4*(1+J19)</f>
         <v/>
       </c>
     </row>
@@ -5666,23 +5666,23 @@
         <v/>
       </c>
       <c r="F6" s="276">
-        <f>E6*(1+F18)</f>
+        <f>E6*(1+F20)</f>
         <v/>
       </c>
       <c r="G6" s="276">
-        <f>F6*(1+G18)</f>
+        <f>F6*(1+G20)</f>
         <v/>
       </c>
       <c r="H6" s="276">
-        <f>G6*(1+H18)</f>
+        <f>G6*(1+H20)</f>
         <v/>
       </c>
       <c r="I6" s="276">
-        <f>H6*(1+I18)</f>
+        <f>H6*(1+I20)</f>
         <v/>
       </c>
       <c r="J6" s="276">
-        <f>I6*(1+J18)</f>
+        <f>I6*(1+J20)</f>
         <v/>
       </c>
     </row>
@@ -5702,23 +5702,23 @@
         <v>14.4</v>
       </c>
       <c r="F7" s="276">
-        <f>E20+0.5*F19</f>
+        <f>E22+0.5*F21</f>
         <v/>
       </c>
       <c r="G7" s="276">
-        <f>F20+0.5*G19</f>
+        <f>F22+0.5*G21</f>
         <v/>
       </c>
       <c r="H7" s="276">
-        <f>G20+0.5*H19</f>
+        <f>G22+0.5*H21</f>
         <v/>
       </c>
       <c r="I7" s="276">
-        <f>H20+0.5*I19</f>
+        <f>H22+0.5*I21</f>
         <v/>
       </c>
       <c r="J7" s="276">
-        <f>I20+0.5*J19</f>
+        <f>I22+0.5*J21</f>
         <v/>
       </c>
     </row>
@@ -5729,35 +5729,35 @@
         </is>
       </c>
       <c r="C8" s="274">
-        <f>C9*C21</f>
+        <f>C9*C23</f>
         <v/>
       </c>
       <c r="D8" s="274">
-        <f>D9*D21</f>
+        <f>D9*D23</f>
         <v/>
       </c>
       <c r="E8" s="275">
-        <f>E9*E21</f>
+        <f>E9*E23</f>
         <v/>
       </c>
       <c r="F8" s="276">
-        <f>(F4+F5)*F21/(1-F21)</f>
+        <f>(F4+F5)*F23/(1-F23)</f>
         <v/>
       </c>
       <c r="G8" s="276">
-        <f>(G4+G5)*G21/(1-G21)</f>
+        <f>(G4+G5)*G23/(1-G23)</f>
         <v/>
       </c>
       <c r="H8" s="276">
-        <f>(H4+H5)*H21/(1-H21)</f>
+        <f>(H4+H5)*H23/(1-H23)</f>
         <v/>
       </c>
       <c r="I8" s="276">
-        <f>(I4+I5)*I21/(1-I21)</f>
+        <f>(I4+I5)*I23/(1-I23)</f>
         <v/>
       </c>
       <c r="J8" s="276">
-        <f>(J4+J5)*J21/(1-J21)</f>
+        <f>(J4+J5)*J23/(1-J23)</f>
         <v/>
       </c>
     </row>
@@ -5963,445 +5963,517 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="12.75" customHeight="1"/>
+    <row r="15" ht="12.75" customHeight="1">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Network deals % of revenue</t>
+        </is>
+      </c>
+      <c r="C15" s="259">
+        <f>C7/C9</f>
+        <v/>
+      </c>
+      <c r="D15" s="259">
+        <f>D7/D9</f>
+        <v/>
+      </c>
+      <c r="E15" s="260">
+        <f>E7/E9</f>
+        <v/>
+      </c>
+      <c r="F15" s="292">
+        <f>F7/F9</f>
+        <v/>
+      </c>
+      <c r="G15" s="292">
+        <f>G7/G9</f>
+        <v/>
+      </c>
+      <c r="H15" s="292">
+        <f>H7/H9</f>
+        <v/>
+      </c>
+      <c r="I15" s="292">
+        <f>I7/I9</f>
+        <v/>
+      </c>
+      <c r="J15" s="292">
+        <f>J7/J9</f>
+        <v/>
+      </c>
+    </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="B16" s="79" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Network deals share of revenue growth</t>
+        </is>
+      </c>
+      <c r="C16" s="259" t="n"/>
+      <c r="D16" s="259">
+        <f>(D7-C7)/(D9-C9)</f>
+        <v/>
+      </c>
+      <c r="E16" s="260">
+        <f>(E7-D7)/(E9-D9)</f>
+        <v/>
+      </c>
+      <c r="F16" s="292">
+        <f>(F7-E7)/(F9-E9)</f>
+        <v/>
+      </c>
+      <c r="G16" s="292">
+        <f>(G7-F7)/(G9-F9)</f>
+        <v/>
+      </c>
+      <c r="H16" s="292">
+        <f>(H7-G7)/(H9-G9)</f>
+        <v/>
+      </c>
+      <c r="I16" s="292">
+        <f>(I7-H7)/(I9-H9)</f>
+        <v/>
+      </c>
+      <c r="J16" s="292">
+        <f>(J7-I7)/(J9-I9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="12.75" customFormat="1" customHeight="1" s="8"/>
+    <row r="18" ht="12.75" customHeight="1">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>DRIVERS</t>
         </is>
       </c>
-      <c r="C16" s="293" t="n"/>
-      <c r="D16" s="294" t="n"/>
-      <c r="E16" s="295" t="n"/>
-      <c r="F16" s="296" t="n"/>
-      <c r="G16" s="296" t="n"/>
-      <c r="H16" s="296" t="n"/>
-      <c r="I16" s="296" t="n"/>
-      <c r="J16" s="296" t="n"/>
-    </row>
-    <row r="17" ht="12.75" customFormat="1" customHeight="1" s="8">
-      <c r="B17" s="85" t="inlineStr">
-        <is>
-          <t>Software revenue % growth</t>
-        </is>
-      </c>
-      <c r="C17" s="297" t="n"/>
-      <c r="D17" s="297">
-        <f>D4/C4-1</f>
-        <v/>
-      </c>
-      <c r="E17" s="298">
-        <f>E4/D4-1</f>
-        <v/>
-      </c>
-      <c r="F17" s="299" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="G17" s="300" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H17" s="300" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I17" s="300" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="J17" s="301" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="18" ht="12.75" customHeight="1">
-      <c r="B18" s="85" t="inlineStr">
-        <is>
-          <t>Microtransit &amp; paratransit % growth (net of downsell)</t>
-        </is>
-      </c>
-      <c r="C18" s="297" t="n"/>
-      <c r="D18" s="297">
-        <f>D6/C6-1</f>
-        <v/>
-      </c>
-      <c r="E18" s="298">
-        <f>E6/D6-1</f>
-        <v/>
-      </c>
-      <c r="F18" s="299" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="G18" s="300" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H18" s="300" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I18" s="300" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="J18" s="301" t="n">
-        <v>0.11</v>
-      </c>
+      <c r="C18" s="293" t="n"/>
+      <c r="D18" s="294" t="n"/>
+      <c r="E18" s="295" t="n"/>
+      <c r="F18" s="296" t="n"/>
+      <c r="G18" s="296" t="n"/>
+      <c r="H18" s="296" t="n"/>
+      <c r="I18" s="296" t="n"/>
+      <c r="J18" s="296" t="n"/>
     </row>
     <row r="19" ht="12.75" customHeight="1">
       <c r="B19" s="85" t="inlineStr">
         <is>
-          <t>Network: new contract value launched ($mm)</t>
-        </is>
-      </c>
-      <c r="C19" s="302" t="n"/>
-      <c r="D19" s="302">
-        <f>D20-C20</f>
-        <v/>
-      </c>
-      <c r="E19" s="303">
-        <f>E20-D20</f>
-        <v/>
-      </c>
-      <c r="F19" s="304" t="n">
-        <v>20</v>
-      </c>
-      <c r="G19" s="305" t="n">
-        <v>30</v>
-      </c>
-      <c r="H19" s="305" t="n">
-        <v>20</v>
-      </c>
-      <c r="I19" s="305" t="n">
-        <v>20</v>
-      </c>
-      <c r="J19" s="306" t="n">
-        <v>20</v>
+          <t>Software revenue % growth</t>
+        </is>
+      </c>
+      <c r="C19" s="297" t="n"/>
+      <c r="D19" s="297">
+        <f>D4/C4-1</f>
+        <v/>
+      </c>
+      <c r="E19" s="298">
+        <f>E4/D4-1</f>
+        <v/>
+      </c>
+      <c r="F19" s="299" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G19" s="300" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H19" s="300" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I19" s="300" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="J19" s="301" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="20" ht="12.75" customHeight="1">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Network: contract run-rate, year-end ($mm)</t>
-        </is>
-      </c>
-      <c r="C20" s="307" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="307" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="E20" s="308" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="F20" s="302">
-        <f>E20+F19</f>
-        <v/>
-      </c>
-      <c r="G20" s="302">
-        <f>F20+G19</f>
-        <v/>
-      </c>
-      <c r="H20" s="302">
-        <f>G20+H19</f>
-        <v/>
-      </c>
-      <c r="I20" s="302">
-        <f>H20+I19</f>
-        <v/>
-      </c>
-      <c r="J20" s="302">
-        <f>I20+J19</f>
-        <v/>
+      <c r="B20" s="85" t="inlineStr">
+        <is>
+          <t>Microtransit &amp; paratransit % growth (net of downsell)</t>
+        </is>
+      </c>
+      <c r="C20" s="297" t="n"/>
+      <c r="D20" s="297">
+        <f>D6/C6-1</f>
+        <v/>
+      </c>
+      <c r="E20" s="298">
+        <f>E6/D6-1</f>
+        <v/>
+      </c>
+      <c r="F20" s="299" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G20" s="300" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H20" s="300" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I20" s="300" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J20" s="301" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="21" ht="12.75" customFormat="1" customHeight="1" s="29">
       <c r="B21" s="85" t="inlineStr">
         <is>
-          <t>One-time revenue % of total</t>
-        </is>
-      </c>
-      <c r="C21" s="309" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D21" s="309" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E21" s="223" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F21" s="299" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="G21" s="300" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="H21" s="300" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="I21" s="300" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="J21" s="301" t="n">
-        <v>0.03</v>
+          <t>Network: new contract value launched ($mm)</t>
+        </is>
+      </c>
+      <c r="C21" s="302" t="n"/>
+      <c r="D21" s="302">
+        <f>D22-C22</f>
+        <v/>
+      </c>
+      <c r="E21" s="303">
+        <f>E22-D22</f>
+        <v/>
+      </c>
+      <c r="F21" s="304" t="n">
+        <v>20</v>
+      </c>
+      <c r="G21" s="305" t="n">
+        <v>40</v>
+      </c>
+      <c r="H21" s="305" t="n">
+        <v>60</v>
+      </c>
+      <c r="I21" s="305" t="n">
+        <v>70</v>
+      </c>
+      <c r="J21" s="306" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="22" ht="12.75" customHeight="1">
       <c r="A22" s="29" t="n"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Network: contract run-rate, year-end ($mm)</t>
+        </is>
+      </c>
+      <c r="C22" s="307" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="307" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E22" s="308" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F22" s="302">
+        <f>E22+F21</f>
+        <v/>
+      </c>
+      <c r="G22" s="302">
+        <f>F22+G21</f>
+        <v/>
+      </c>
+      <c r="H22" s="302">
+        <f>G22+H21</f>
+        <v/>
+      </c>
+      <c r="I22" s="302">
+        <f>H22+I21</f>
+        <v/>
+      </c>
+      <c r="J22" s="302">
+        <f>I22+J21</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="12.75" customHeight="1">
       <c r="A23" s="29" t="n"/>
-      <c r="B23" s="84" t="inlineStr">
+      <c r="B23" s="85" t="inlineStr">
+        <is>
+          <t>One-time revenue % of total</t>
+        </is>
+      </c>
+      <c r="C23" s="309" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D23" s="309" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E23" s="223" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F23" s="299" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G23" s="300" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H23" s="300" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I23" s="300" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J23" s="301" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="24" ht="12.75" customHeight="1"/>
+    <row r="25" ht="12.75" customHeight="1">
+      <c r="B25" s="84" t="inlineStr">
         <is>
           <t>GROSS MARGIN BY STREAM</t>
         </is>
       </c>
-      <c r="C23" s="310" t="n"/>
-      <c r="D23" s="310" t="n"/>
-      <c r="E23" s="311" t="n"/>
-      <c r="F23" s="312" t="n"/>
-      <c r="G23" s="312" t="n"/>
-      <c r="H23" s="312" t="n"/>
-      <c r="I23" s="312" t="n"/>
-      <c r="J23" s="312" t="n"/>
-    </row>
-    <row r="24" ht="12.75" customHeight="1">
-      <c r="B24" s="85" t="inlineStr">
-        <is>
-          <t>Software</t>
-        </is>
-      </c>
-      <c r="C24" s="297" t="n"/>
-      <c r="D24" s="297" t="n"/>
-      <c r="E24" s="298" t="n"/>
-      <c r="F24" s="299" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G24" s="300" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H24" s="300" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I24" s="300" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J24" s="301" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="25" ht="12.75" customHeight="1">
-      <c r="B25" s="85" t="inlineStr">
-        <is>
-          <t>Microtransit &amp; paratransit</t>
-        </is>
-      </c>
-      <c r="C25" s="297" t="n"/>
-      <c r="D25" s="297" t="n"/>
-      <c r="E25" s="298" t="n"/>
-      <c r="F25" s="299" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="G25" s="300" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="H25" s="300" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="I25" s="300" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="J25" s="301" t="n">
-        <v>0.293</v>
-      </c>
+      <c r="C25" s="310" t="n"/>
+      <c r="D25" s="310" t="n"/>
+      <c r="E25" s="311" t="n"/>
+      <c r="F25" s="312" t="n"/>
+      <c r="G25" s="312" t="n"/>
+      <c r="H25" s="312" t="n"/>
+      <c r="I25" s="312" t="n"/>
+      <c r="J25" s="312" t="n"/>
     </row>
     <row r="26" ht="12.75" customFormat="1" customHeight="1" s="29">
       <c r="B26" s="85" t="inlineStr">
         <is>
-          <t>Network deals</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C26" s="297" t="n"/>
       <c r="D26" s="297" t="n"/>
       <c r="E26" s="298" t="n"/>
       <c r="F26" s="299" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="G26" s="300" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="H26" s="300" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="I26" s="300" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="J26" s="301" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="27" ht="12.75" customHeight="1">
       <c r="A27" s="29" t="n"/>
       <c r="B27" s="85" t="inlineStr">
         <is>
-          <t>One-time</t>
+          <t>Microtransit &amp; paratransit</t>
         </is>
       </c>
       <c r="C27" s="297" t="n"/>
       <c r="D27" s="297" t="n"/>
       <c r="E27" s="298" t="n"/>
       <c r="F27" s="299" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="G27" s="300" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="H27" s="300" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="I27" s="300" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="J27" s="301" t="n">
+        <v>0.293</v>
+      </c>
+    </row>
+    <row r="28" ht="12.75" customFormat="1" customHeight="1" s="29">
+      <c r="B28" s="85" t="inlineStr">
+        <is>
+          <t>Network deals</t>
+        </is>
+      </c>
+      <c r="C28" s="297" t="n"/>
+      <c r="D28" s="297" t="n"/>
+      <c r="E28" s="298" t="n"/>
+      <c r="F28" s="299" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G28" s="300" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H28" s="300" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I28" s="300" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J28" s="301" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="29" ht="12.75" customFormat="1" customHeight="1" s="29">
+      <c r="B29" s="85" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="C29" s="297" t="n"/>
+      <c r="D29" s="297" t="n"/>
+      <c r="E29" s="298" t="n"/>
+      <c r="F29" s="299" t="n">
         <v>0.75</v>
       </c>
-      <c r="G27" s="300" t="n">
+      <c r="G29" s="300" t="n">
         <v>0.75</v>
       </c>
-      <c r="H27" s="300" t="n">
+      <c r="H29" s="300" t="n">
         <v>0.75</v>
       </c>
-      <c r="I27" s="300" t="n">
+      <c r="I29" s="300" t="n">
         <v>0.75</v>
       </c>
-      <c r="J27" s="301" t="n">
+      <c r="J29" s="301" t="n">
         <v>0.75</v>
       </c>
     </row>
-    <row r="28" ht="12.75" customFormat="1" customHeight="1" s="29">
-      <c r="B28" s="26" t="inlineStr">
+    <row r="30" ht="12.75" customHeight="1">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>Gross profit ($mm)</t>
         </is>
       </c>
-      <c r="C28" s="278">
+      <c r="C30" s="278">
         <f>'Annual IS'!B10</f>
         <v/>
       </c>
-      <c r="D28" s="278">
+      <c r="D30" s="278">
         <f>'Annual IS'!C10</f>
         <v/>
       </c>
-      <c r="E28" s="279">
+      <c r="E30" s="279">
         <f>'Annual IS'!D10</f>
         <v/>
       </c>
-      <c r="F28" s="277">
-        <f>F4*F24+F6*F25+F7*F26+F8*F27</f>
-        <v/>
-      </c>
-      <c r="G28" s="277">
-        <f>G4*G24+G6*G25+G7*G26+G8*G27</f>
-        <v/>
-      </c>
-      <c r="H28" s="277">
-        <f>H4*H24+H6*H25+H7*H26+H8*H27</f>
-        <v/>
-      </c>
-      <c r="I28" s="277">
-        <f>I4*I24+I6*I25+I7*I26+I8*I27</f>
-        <v/>
-      </c>
-      <c r="J28" s="277">
-        <f>J4*J24+J6*J25+J7*J26+J8*J27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="12.75" customFormat="1" customHeight="1" s="29">
-      <c r="B29" s="280" t="inlineStr">
+      <c r="F30" s="277">
+        <f>F4*F26+F6*F27+F7*F28+F8*F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="277">
+        <f>G4*G26+G6*G27+G7*G28+G8*G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="277">
+        <f>H4*H26+H6*H27+H7*H28+H8*H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="277">
+        <f>I4*I26+I6*I27+I7*I28+I8*I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="277">
+        <f>J4*J26+J6*J27+J7*J28+J8*J29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="12.75" customHeight="1">
+      <c r="B31" s="280" t="inlineStr">
         <is>
           <t xml:space="preserve">   Gross margin</t>
         </is>
       </c>
-      <c r="C29" s="281">
-        <f>C28/C9</f>
-        <v/>
-      </c>
-      <c r="D29" s="282">
-        <f>D28/D9</f>
-        <v/>
-      </c>
-      <c r="E29" s="283">
-        <f>E28/E9</f>
-        <v/>
-      </c>
-      <c r="F29" s="282">
-        <f>F28/F9</f>
-        <v/>
-      </c>
-      <c r="G29" s="282">
-        <f>G28/G9</f>
-        <v/>
-      </c>
-      <c r="H29" s="282">
-        <f>H28/H9</f>
-        <v/>
-      </c>
-      <c r="I29" s="282">
-        <f>I28/I9</f>
-        <v/>
-      </c>
-      <c r="J29" s="282">
-        <f>J28/J9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="12.75" customHeight="1">
-      <c r="B30" s="288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Consensus gross margin (BBG; FY28 CapIQ)</t>
-        </is>
-      </c>
-      <c r="C30" s="289">
-        <f>C29</f>
-        <v/>
-      </c>
-      <c r="D30" s="289">
-        <f>D29</f>
-        <v/>
-      </c>
-      <c r="E30" s="290">
-        <f>E29</f>
-        <v/>
-      </c>
-      <c r="F30" s="313">
-        <f>'Consensus (BBG)'!P23</f>
-        <v/>
-      </c>
-      <c r="G30" s="313">
-        <f>'Consensus (BBG)'!Q23</f>
-        <v/>
-      </c>
-      <c r="H30" s="313">
-        <f>'Key Stats'!H20</f>
-        <v/>
-      </c>
-      <c r="I30" s="291" t="n"/>
-      <c r="J30" s="291" t="n"/>
-    </row>
-    <row r="31" ht="12.75" customHeight="1"/>
+      <c r="C31" s="281">
+        <f>C30/C9</f>
+        <v/>
+      </c>
+      <c r="D31" s="282">
+        <f>D30/D9</f>
+        <v/>
+      </c>
+      <c r="E31" s="283">
+        <f>E30/E9</f>
+        <v/>
+      </c>
+      <c r="F31" s="282">
+        <f>F30/F9</f>
+        <v/>
+      </c>
+      <c r="G31" s="282">
+        <f>G30/G9</f>
+        <v/>
+      </c>
+      <c r="H31" s="282">
+        <f>H30/H9</f>
+        <v/>
+      </c>
+      <c r="I31" s="282">
+        <f>I30/I9</f>
+        <v/>
+      </c>
+      <c r="J31" s="282">
+        <f>J30/J9</f>
+        <v/>
+      </c>
+    </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="29" t="n"/>
-      <c r="B32" s="314" t="inlineStr">
-        <is>
-          <t>Colour key: blue = hardcoded input, black = formula, green = link to another tab. Hover over cells with a red corner for sources.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="12.75" customFormat="1" customHeight="1" s="29">
-      <c r="B33" s="314" t="inlineStr">
-        <is>
-          <t>Thesis 1: network deals are bus-operator contracts priced at ~95-107% of the city's transit budget, so they carry a 25% gross margin vs ~29% on microtransit and 75% on software.</t>
-        </is>
-      </c>
-    </row>
+      <c r="B32" s="288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consensus gross margin (BBG; FY28 CapIQ)</t>
+        </is>
+      </c>
+      <c r="C32" s="289">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="D32" s="289">
+        <f>D31</f>
+        <v/>
+      </c>
+      <c r="E32" s="290">
+        <f>E31</f>
+        <v/>
+      </c>
+      <c r="F32" s="313">
+        <f>'Consensus (BBG)'!P23</f>
+        <v/>
+      </c>
+      <c r="G32" s="313">
+        <f>'Consensus (BBG)'!Q23</f>
+        <v/>
+      </c>
+      <c r="H32" s="313">
+        <f>'Key Stats'!H20</f>
+        <v/>
+      </c>
+      <c r="I32" s="291" t="n"/>
+      <c r="J32" s="291" t="n"/>
+    </row>
+    <row r="33" ht="12.75" customFormat="1" customHeight="1" s="29"/>
     <row r="34" ht="12.75" customHeight="1">
       <c r="B34" s="314" t="inlineStr">
         <is>
-          <t>Thesis 3: microtransit/paratransit growth is net of budget-driven downsell and rebid price resets.</t>
+          <t>Colour key: blue = hardcoded input, black = formula, green = link to another tab. Hover over cells with a red corner for sources.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="B35" s="314" t="inlineStr">
         <is>
+          <t>Thesis 1: network deals are bus-operator contracts priced at ~95-107% of the city's transit budget, so they carry a 25% gross margin vs ~29% on microtransit and 75% on software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="12.75" customHeight="1">
+      <c r="B36" s="314" t="inlineStr">
+        <is>
+          <t>Thesis 1: network deals become the growth engine (~a third of FY27 growth, ~25% of revenue by FY30), dragging gross margin toward operator levels. Thesis 3: microtransit/paratransit growth is net of budget-driven downsell and rebid price resets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="12.75" customHeight="1">
+      <c r="B37" s="314" t="inlineStr">
+        <is>
           <t>Consensus: Bloomberg FY26-27E (Consensus (BBG) tab, sum of quarters); FY28E from CapIQ (Key Stats tab) because Bloomberg stops at Q4 2027. FY29-30 have no consensus.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="12.75" customHeight="1"/>
-    <row r="37" ht="12.75" customHeight="1"/>
     <row r="38" ht="12.75" customHeight="1"/>
     <row r="39" ht="12.75" customHeight="1"/>
     <row r="40" ht="12.75" customHeight="1"/>
@@ -6438,9 +6510,9 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C2:E2"/>
-    <mergeCell ref="B33:J33"/>
     <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B36:J36"/>
     <mergeCell ref="B35:J35"/>
     <mergeCell ref="F2:J2"/>
   </mergeCells>

</xml_diff>